<commit_message>
Worked on Excel file and matrices Signed-off-by: Student Harvey Smith (TL_KCOMP_B_Y3) <t00264389@mymtu.ie>
</commit_message>
<xml_diff>
--- a/Computer Graphics/ASSIGNMENT XL.xlsx
+++ b/Computer Graphics/ASSIGNMENT XL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StudentHarveySmith(T\Desktop\CG\Computer Graphics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StudentHarveySmith(T\Desktop\ComputerG\Computer Graphics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{30EAB396-942C-47F1-9DC8-364E3EC6A77E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B748EAE3-64DD-462A-A8E4-0959F694A320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -559,44 +559,44 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -843,22 +843,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>734786</xdr:colOff>
+      <xdr:colOff>455544</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>68036</xdr:rowOff>
+      <xdr:rowOff>48702</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
+      <xdr:colOff>727231</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>1317226</xdr:rowOff>
+      <xdr:rowOff>1320032</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="Picture 10">
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1BA5C403-FB1C-D9A5-5D84-4A8775A20506}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{624B4747-6B34-1935-E044-E681AD75FADF}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -874,8 +874,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2571750" y="20655643"/>
-          <a:ext cx="2054679" cy="1249190"/>
+          <a:off x="2294283" y="20655832"/>
+          <a:ext cx="2773035" cy="1271330"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -887,22 +887,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>975329</xdr:colOff>
+      <xdr:colOff>140239</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:rowOff>74543</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>136071</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1935220</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>5122132</xdr:rowOff>
+      <xdr:rowOff>5016647</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Picture 11">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{62381632-C1DC-6A02-6CAD-8D0C4A34DF43}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5958AB2E-FC7C-D6B1-E0FD-B38E5A7BCCAB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -918,8 +918,360 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2812293" y="22370143"/>
-          <a:ext cx="1664457" cy="5026882"/>
+          <a:off x="1978978" y="22371326"/>
+          <a:ext cx="1794981" cy="4942104"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1962980</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>1674726</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1192696</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>2084411</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{02E901EE-39DB-6887-0280-AD12EDA32468}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3801719" y="23971509"/>
+          <a:ext cx="1731064" cy="409685"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>488674</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>180425</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>597593</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>1073618</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{79624E3F-F4E5-F45E-3963-89E44C1783EA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8680174" y="13739055"/>
+          <a:ext cx="1947658" cy="893193"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>57978</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>49695</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>757859</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>5126934</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Picture 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{01077B1D-53A1-D655-BEEA-30E46C1EE6E0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8249478" y="22346478"/>
+          <a:ext cx="2538620" cy="5077239"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>560294</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>78442</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>257736</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>1349704</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="18" name="Picture 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0984A5F5-7C18-07B6-5799-49E5256DD903}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12315265" y="27756971"/>
+          <a:ext cx="2577353" cy="1271262"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>680357</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>81644</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>802821</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>1343904</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="Picture 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{47F83352-7530-3D09-6359-0DD23B4AB7A4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2517321" y="27881037"/>
+          <a:ext cx="2626179" cy="1262260"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>875586</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>40822</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>547519</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>5068486</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="21" name="Picture 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{01D17FC9-A63F-9265-D2D2-D643F84E8F5E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2712550" y="29609143"/>
+          <a:ext cx="2175648" cy="5027664"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>489857</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>1129393</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>920251</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>2577395</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="22" name="Picture 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1AF54C60-25ED-C67B-B26F-3C0DC1FF7AC6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2326821" y="36222214"/>
+          <a:ext cx="2934109" cy="1448002"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1161692</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>197550</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>231320</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>4854854</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="23" name="Picture 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5DC7135F-D495-0E10-406B-AB588FE17722}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2998656" y="39712693"/>
+          <a:ext cx="1573343" cy="4657304"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1231,24 +1583,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
     </row>
     <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
     </row>
     <row r="3" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -1613,7 +1965,7 @@
   <cols>
     <col min="1" max="3" width="9.140625" customWidth="1"/>
     <col min="4" max="4" width="37.5703125" customWidth="1"/>
-    <col min="5" max="5" width="19" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="21" customWidth="1"/>
     <col min="7" max="7" width="17.7109375" customWidth="1"/>
     <col min="8" max="8" width="27.5703125" customWidth="1"/>
@@ -1630,10 +1982,10 @@
     </row>
     <row r="2" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C2" s="4"/>
-      <c r="D2" s="42" t="s">
+      <c r="D2" s="46" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="43"/>
+      <c r="E2" s="47"/>
       <c r="F2" s="7"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
@@ -1644,8 +1996,8 @@
     </row>
     <row r="3" spans="3:13" ht="408.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C3" s="4"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="41"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="40"/>
       <c r="F3" s="5"/>
       <c r="G3" s="10"/>
       <c r="H3" s="6"/>
@@ -1665,10 +2017,10 @@
     </row>
     <row r="5" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C5" s="4"/>
-      <c r="D5" s="42" t="s">
+      <c r="D5" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="43"/>
+      <c r="E5" s="47"/>
       <c r="F5" s="7"/>
       <c r="H5" s="14"/>
       <c r="I5" s="11"/>
@@ -1677,8 +2029,8 @@
     </row>
     <row r="6" spans="3:13" ht="138.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C6" s="4"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="41"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="40"/>
       <c r="F6" s="15"/>
       <c r="G6" s="11"/>
       <c r="H6" s="14"/>
@@ -1698,10 +2050,10 @@
     </row>
     <row r="8" spans="3:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C8" s="4"/>
-      <c r="D8" s="42" t="s">
+      <c r="D8" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="43"/>
+      <c r="E8" s="47"/>
       <c r="F8" s="16"/>
       <c r="G8" s="11"/>
       <c r="H8" s="14"/>
@@ -1711,8 +2063,8 @@
     </row>
     <row r="9" spans="3:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C9" s="4"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="41"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="40"/>
       <c r="F9" s="16"/>
       <c r="G9" s="11"/>
       <c r="H9" s="14"/>
@@ -1732,10 +2084,10 @@
     </row>
     <row r="11" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C11" s="4"/>
-      <c r="D11" s="42" t="s">
+      <c r="D11" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="43"/>
+      <c r="E11" s="47"/>
       <c r="F11" s="17"/>
       <c r="G11" s="18"/>
       <c r="H11" s="44" t="s">
@@ -1748,12 +2100,12 @@
     </row>
     <row r="12" spans="3:13" ht="93" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C12" s="4"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="41"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="40"/>
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
-      <c r="H12" s="40"/>
-      <c r="I12" s="41"/>
+      <c r="H12" s="38"/>
+      <c r="I12" s="40"/>
       <c r="J12" s="15"/>
       <c r="K12" s="11"/>
       <c r="L12" s="14"/>
@@ -1773,10 +2125,10 @@
     </row>
     <row r="14" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C14" s="4"/>
-      <c r="D14" s="42" t="s">
+      <c r="D14" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="43"/>
+      <c r="E14" s="47"/>
       <c r="F14" s="16"/>
       <c r="G14" s="11"/>
       <c r="H14" s="14"/>
@@ -1788,8 +2140,8 @@
     </row>
     <row r="15" spans="3:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C15" s="4"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="41"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="40"/>
       <c r="F15" s="16"/>
       <c r="G15" s="11"/>
       <c r="H15" s="14"/>
@@ -1813,10 +2165,10 @@
     </row>
     <row r="17" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C17" s="4"/>
-      <c r="D17" s="42" t="s">
+      <c r="D17" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="E17" s="43"/>
+      <c r="E17" s="47"/>
       <c r="F17" s="17"/>
       <c r="G17" s="11"/>
       <c r="H17" s="14"/>
@@ -1828,8 +2180,8 @@
     </row>
     <row r="18" spans="1:13" ht="107.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C18" s="4"/>
-      <c r="D18" s="40"/>
-      <c r="E18" s="41"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="40"/>
       <c r="F18" s="19"/>
       <c r="H18" s="14"/>
       <c r="I18" s="11"/>
@@ -1850,14 +2202,14 @@
     </row>
     <row r="20" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C20" s="4"/>
-      <c r="D20" s="42" t="s">
+      <c r="D20" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="E20" s="43"/>
-      <c r="F20" s="46" t="s">
+      <c r="E20" s="47"/>
+      <c r="F20" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="G20" s="47"/>
+      <c r="G20" s="43"/>
       <c r="H20" s="44" t="s">
         <v>1</v>
       </c>
@@ -1869,12 +2221,12 @@
     </row>
     <row r="21" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C21" s="4"/>
-      <c r="D21" s="40"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="46"/>
-      <c r="G21" s="47"/>
-      <c r="H21" s="40"/>
-      <c r="I21" s="41"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="38"/>
+      <c r="I21" s="40"/>
       <c r="J21" s="16"/>
       <c r="K21" s="11"/>
       <c r="L21" s="14"/>
@@ -1892,10 +2244,10 @@
     </row>
     <row r="23" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C23" s="4"/>
-      <c r="D23" s="42" t="s">
+      <c r="D23" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="E23" s="43"/>
+      <c r="E23" s="47"/>
       <c r="F23" s="8"/>
       <c r="G23" s="21"/>
       <c r="H23" s="21"/>
@@ -1909,16 +2261,16 @@
     </row>
     <row r="24" spans="1:13" ht="113.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C24" s="4"/>
-      <c r="D24" s="40"/>
-      <c r="E24" s="41"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="40"/>
       <c r="F24" s="5"/>
       <c r="G24" s="10"/>
       <c r="H24" s="10"/>
       <c r="I24" s="10"/>
       <c r="J24" s="6"/>
       <c r="K24" s="22"/>
-      <c r="L24" s="40"/>
-      <c r="M24" s="41"/>
+      <c r="L24" s="38"/>
+      <c r="M24" s="40"/>
     </row>
     <row r="25" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D25" s="12"/>
@@ -1945,8 +2297,8 @@
       <c r="A27" s="4"/>
       <c r="B27" s="5"/>
       <c r="C27" s="6"/>
-      <c r="D27" s="40"/>
-      <c r="E27" s="41"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="40"/>
       <c r="F27" s="11"/>
       <c r="J27" s="14"/>
       <c r="K27" s="11"/>
@@ -1969,10 +2321,10 @@
       </c>
       <c r="B29" s="45"/>
       <c r="C29" s="24"/>
-      <c r="D29" s="42" t="s">
+      <c r="D29" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="43"/>
+      <c r="E29" s="47"/>
       <c r="F29" s="8"/>
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
@@ -1983,11 +2335,11 @@
       <c r="M29" s="11"/>
     </row>
     <row r="30" spans="1:13" ht="322.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="40"/>
-      <c r="B30" s="41"/>
+      <c r="A30" s="38"/>
+      <c r="B30" s="40"/>
       <c r="C30" s="24"/>
-      <c r="D30" s="40"/>
-      <c r="E30" s="41"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="40"/>
       <c r="F30" s="19"/>
       <c r="G30" s="20"/>
       <c r="H30" s="20"/>
@@ -2005,44 +2357,44 @@
       <c r="M31" s="7"/>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A32" s="42" t="s">
+      <c r="A32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B32" s="43"/>
+      <c r="B32" s="47"/>
       <c r="C32" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="42" t="s">
+      <c r="D32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="E32" s="43"/>
-      <c r="F32" s="46" t="s">
+      <c r="E32" s="47"/>
+      <c r="F32" s="41" t="s">
         <v>31</v>
       </c>
-      <c r="G32" s="49"/>
-      <c r="H32" s="49"/>
-      <c r="I32" s="49"/>
-      <c r="J32" s="49"/>
-      <c r="K32" s="47"/>
-      <c r="L32" s="42" t="s">
+      <c r="G32" s="42"/>
+      <c r="H32" s="42"/>
+      <c r="I32" s="42"/>
+      <c r="J32" s="42"/>
+      <c r="K32" s="43"/>
+      <c r="L32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="M32" s="43"/>
-    </row>
-    <row r="33" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="50"/>
-      <c r="B33" s="48"/>
+      <c r="M32" s="47"/>
+    </row>
+    <row r="33" spans="1:13" ht="394.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="48"/>
+      <c r="B33" s="39"/>
       <c r="C33" s="16"/>
-      <c r="D33" s="40"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="46"/>
-      <c r="G33" s="49"/>
-      <c r="H33" s="49"/>
-      <c r="I33" s="49"/>
-      <c r="J33" s="49"/>
-      <c r="K33" s="47"/>
-      <c r="L33" s="40"/>
-      <c r="M33" s="48"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="40"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="42"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="42"/>
+      <c r="J33" s="42"/>
+      <c r="K33" s="43"/>
+      <c r="L33" s="38"/>
+      <c r="M33" s="39"/>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="20"/>
@@ -2062,38 +2414,25 @@
     </row>
     <row r="36" spans="1:13" ht="213.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C36" s="4"/>
-      <c r="D36" s="40"/>
-      <c r="E36" s="41"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="40"/>
       <c r="F36" s="11"/>
     </row>
     <row r="38" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E38" s="25"/>
       <c r="F38" s="25"/>
-      <c r="H38" s="40"/>
-      <c r="I38" s="48"/>
+      <c r="H38" s="38"/>
+      <c r="I38" s="39"/>
     </row>
     <row r="91" ht="0.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="H38:I38"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="F32:K32"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="F33:K33"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="L23:M23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="L24:M24"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="L32:M32"/>
-    <mergeCell ref="L33:M33"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D8:E8"/>
     <mergeCell ref="H20:I20"/>
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="H11:I11"/>
@@ -2110,12 +2449,25 @@
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="L23:M23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="L32:M32"/>
+    <mergeCell ref="L33:M33"/>
+    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="F32:K32"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="F33:K33"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="D32:E32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Fixed small issues and now have matrices correct and matching Signed-off-by: Harvey <HarveyDanSmith@gmail.com>
</commit_message>
<xml_diff>
--- a/Computer Graphics/ASSIGNMENT XL.xlsx
+++ b/Computer Graphics/ASSIGNMENT XL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StudentHarveySmith(T\Desktop\ComputerG\Computer Graphics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Harve\Desktop\CompGraph\Computer Graphics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B748EAE3-64DD-462A-A8E4-0959F694A320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC678811-1534-40A7-9299-74E9DA1DAB42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assignment generation" sheetId="1" r:id="rId1"/>
@@ -563,30 +563,30 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1280,6 +1280,94 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>115002</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>163974</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>2083443</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>4891550</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6BF3BAEF-CAEB-FE46-69B2-2572DAAE632C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12422749" y="39643290"/>
+          <a:ext cx="1968441" cy="4727576"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>2112380</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>1263570</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>917087</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>2633241</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Picture 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{996109CA-8D98-F149-DE4B-FC70E1A7853D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14420127" y="40742886"/>
+          <a:ext cx="1765897" cy="1369671"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1571,18 +1659,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K29"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="46.7109375" customWidth="1"/>
-    <col min="2" max="2" width="22.5703125" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" style="25" customWidth="1"/>
-    <col min="4" max="6" width="9.140625" style="25" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="25"/>
-    <col min="10" max="10" width="16.42578125" style="35" customWidth="1"/>
+    <col min="1" max="1" width="46.6640625" customWidth="1"/>
+    <col min="2" max="2" width="22.5546875" customWidth="1"/>
+    <col min="3" max="3" width="10.88671875" style="25" customWidth="1"/>
+    <col min="4" max="6" width="9.109375" style="25" customWidth="1"/>
+    <col min="7" max="9" width="9.109375" style="25"/>
+    <col min="10" max="10" width="16.44140625" style="35" customWidth="1"/>
     <col min="11" max="11" width="57" style="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="49" t="s">
         <v>19</v>
       </c>
@@ -1592,7 +1680,7 @@
       <c r="E1" s="49"/>
       <c r="F1" s="49"/>
     </row>
-    <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="50" t="s">
         <v>36</v>
       </c>
@@ -1602,12 +1690,12 @@
       <c r="E2" s="50"/>
       <c r="F2" s="50"/>
     </row>
-    <row r="3" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>22</v>
       </c>
@@ -1615,7 +1703,7 @@
         <v>264389</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
@@ -1627,7 +1715,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>23</v>
       </c>
@@ -1665,7 +1753,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -1685,7 +1773,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>26</v>
       </c>
@@ -1705,10 +1793,10 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C10" s="27"/>
     </row>
-    <row r="11" spans="1:10" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>29</v>
       </c>
@@ -1728,7 +1816,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2"/>
       <c r="B12" s="1" t="s">
         <v>9</v>
@@ -1749,7 +1837,7 @@
       <c r="G12" s="37"/>
       <c r="I12" s="37"/>
     </row>
-    <row r="13" spans="1:10" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
         <v>28</v>
@@ -1785,42 +1873,42 @@
         <v>39</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="12.75" hidden="1" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="12.75" hidden="1" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="27"/>
     </row>
-    <row r="15" spans="1:10" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="27"/>
     </row>
-    <row r="16" spans="1:10" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="27"/>
     </row>
-    <row r="17" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="27"/>
     </row>
-    <row r="18" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="27"/>
     </row>
-    <row r="19" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="27"/>
     </row>
-    <row r="20" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="27"/>
     </row>
-    <row r="21" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C21" s="31">
         <f>INT((C4/10000))-5</f>
         <v>21</v>
@@ -1838,7 +1926,7 @@
         <v>21.189620100417091</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C22" s="32">
         <f>MOD(INT((C4/10000)),6) + 1</f>
         <v>3</v>
@@ -1856,7 +1944,7 @@
         <v>7.0710678118654755</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C23" s="27">
         <f>MOD(C4,10)-5</f>
         <v>4</v>
@@ -1874,13 +1962,13 @@
         <v>5.0990195135927845</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G24" s="25">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C25" s="27">
         <f>2+C21</f>
         <v>23</v>
@@ -1898,7 +1986,7 @@
         <v>53.235326616824658</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C26" s="31">
         <f>D21</f>
         <v>-2</v>
@@ -1916,7 +2004,7 @@
         <v>5.3851648071345037</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
       <c r="C27" s="31">
         <f>E23</f>
@@ -1935,8 +2023,8 @@
         <v>21.118712081942874</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="29" spans="1:7" ht="12.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:7" ht="12.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>34</v>
       </c>
@@ -1961,31 +2049,31 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M91"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="9.140625" customWidth="1"/>
-    <col min="4" max="4" width="37.5703125" customWidth="1"/>
+    <col min="1" max="3" width="9.109375" customWidth="1"/>
+    <col min="4" max="4" width="37.5546875" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
     <col min="6" max="6" width="21" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" customWidth="1"/>
-    <col min="8" max="8" width="27.5703125" customWidth="1"/>
-    <col min="9" max="9" width="13.42578125" customWidth="1"/>
-    <col min="10" max="10" width="9.140625" customWidth="1"/>
-    <col min="11" max="11" width="3.7109375" customWidth="1"/>
-    <col min="12" max="12" width="43.140625" customWidth="1"/>
-    <col min="13" max="13" width="14.42578125" customWidth="1"/>
+    <col min="7" max="7" width="17.6640625" customWidth="1"/>
+    <col min="8" max="8" width="27.5546875" customWidth="1"/>
+    <col min="9" max="9" width="13.44140625" customWidth="1"/>
+    <col min="10" max="10" width="9.109375" customWidth="1"/>
+    <col min="11" max="11" width="3.6640625" customWidth="1"/>
+    <col min="12" max="12" width="43.109375" customWidth="1"/>
+    <col min="13" max="13" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
     </row>
-    <row r="2" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C2" s="4"/>
-      <c r="D2" s="46" t="s">
+      <c r="D2" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="47"/>
+      <c r="E2" s="41"/>
       <c r="F2" s="7"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
@@ -1994,10 +2082,10 @@
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
     </row>
-    <row r="3" spans="3:13" ht="408.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="3:13" ht="408.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="4"/>
       <c r="D3" s="38"/>
-      <c r="E3" s="40"/>
+      <c r="E3" s="39"/>
       <c r="F3" s="5"/>
       <c r="G3" s="10"/>
       <c r="H3" s="6"/>
@@ -2007,7 +2095,7 @@
       <c r="L3" s="6"/>
       <c r="M3" s="11"/>
     </row>
-    <row r="4" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D4" s="12"/>
       <c r="E4" s="13"/>
       <c r="H4" s="14"/>
@@ -2015,22 +2103,22 @@
       <c r="L4" s="14"/>
       <c r="M4" s="11"/>
     </row>
-    <row r="5" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C5" s="4"/>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="47"/>
+      <c r="E5" s="41"/>
       <c r="F5" s="7"/>
       <c r="H5" s="14"/>
       <c r="I5" s="11"/>
       <c r="L5" s="14"/>
       <c r="M5" s="11"/>
     </row>
-    <row r="6" spans="3:13" ht="138.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="3:13" ht="138.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C6" s="4"/>
       <c r="D6" s="38"/>
-      <c r="E6" s="40"/>
+      <c r="E6" s="39"/>
       <c r="F6" s="15"/>
       <c r="G6" s="11"/>
       <c r="H6" s="14"/>
@@ -2038,7 +2126,7 @@
       <c r="L6" s="14"/>
       <c r="M6" s="11"/>
     </row>
-    <row r="7" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D7" s="12"/>
       <c r="E7" s="13"/>
       <c r="F7" s="14"/>
@@ -2048,12 +2136,12 @@
       <c r="L7" s="14"/>
       <c r="M7" s="11"/>
     </row>
-    <row r="8" spans="3:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="3:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C8" s="4"/>
-      <c r="D8" s="46" t="s">
+      <c r="D8" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="47"/>
+      <c r="E8" s="41"/>
       <c r="F8" s="16"/>
       <c r="G8" s="11"/>
       <c r="H8" s="14"/>
@@ -2061,10 +2149,10 @@
       <c r="L8" s="14"/>
       <c r="M8" s="11"/>
     </row>
-    <row r="9" spans="3:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="3:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="4"/>
       <c r="D9" s="38"/>
-      <c r="E9" s="40"/>
+      <c r="E9" s="39"/>
       <c r="F9" s="16"/>
       <c r="G9" s="11"/>
       <c r="H9" s="14"/>
@@ -2072,7 +2160,7 @@
       <c r="L9" s="14"/>
       <c r="M9" s="11"/>
     </row>
-    <row r="10" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D10" s="12"/>
       <c r="E10" s="13"/>
       <c r="F10" s="14"/>
@@ -2082,36 +2170,36 @@
       <c r="L10" s="14"/>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C11" s="4"/>
-      <c r="D11" s="46" t="s">
+      <c r="D11" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="47"/>
+      <c r="E11" s="41"/>
       <c r="F11" s="17"/>
       <c r="G11" s="18"/>
-      <c r="H11" s="44" t="s">
+      <c r="H11" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="I11" s="45"/>
+      <c r="I11" s="43"/>
       <c r="J11" s="7"/>
       <c r="L11" s="14"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="3:13" ht="93" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="3:13" ht="93" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C12" s="4"/>
       <c r="D12" s="38"/>
-      <c r="E12" s="40"/>
+      <c r="E12" s="39"/>
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
       <c r="H12" s="38"/>
-      <c r="I12" s="40"/>
+      <c r="I12" s="39"/>
       <c r="J12" s="15"/>
       <c r="K12" s="11"/>
       <c r="L12" s="14"/>
       <c r="M12" s="11"/>
     </row>
-    <row r="13" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D13" s="12"/>
       <c r="E13" s="13"/>
       <c r="F13" s="14"/>
@@ -2123,12 +2211,12 @@
       <c r="L13" s="14"/>
       <c r="M13" s="11"/>
     </row>
-    <row r="14" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C14" s="4"/>
-      <c r="D14" s="46" t="s">
+      <c r="D14" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="47"/>
+      <c r="E14" s="41"/>
       <c r="F14" s="16"/>
       <c r="G14" s="11"/>
       <c r="H14" s="14"/>
@@ -2138,10 +2226,10 @@
       <c r="L14" s="14"/>
       <c r="M14" s="11"/>
     </row>
-    <row r="15" spans="3:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="3:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C15" s="4"/>
       <c r="D15" s="38"/>
-      <c r="E15" s="40"/>
+      <c r="E15" s="39"/>
       <c r="F15" s="16"/>
       <c r="G15" s="11"/>
       <c r="H15" s="14"/>
@@ -2151,7 +2239,7 @@
       <c r="L15" s="14"/>
       <c r="M15" s="11"/>
     </row>
-    <row r="16" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D16" s="12"/>
       <c r="E16" s="13"/>
       <c r="F16" s="14"/>
@@ -2163,12 +2251,12 @@
       <c r="L16" s="14"/>
       <c r="M16" s="11"/>
     </row>
-    <row r="17" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C17" s="4"/>
-      <c r="D17" s="46" t="s">
+      <c r="D17" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="E17" s="47"/>
+      <c r="E17" s="41"/>
       <c r="F17" s="17"/>
       <c r="G17" s="11"/>
       <c r="H17" s="14"/>
@@ -2178,10 +2266,10 @@
       <c r="L17" s="14"/>
       <c r="M17" s="11"/>
     </row>
-    <row r="18" spans="1:13" ht="107.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" ht="107.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C18" s="4"/>
       <c r="D18" s="38"/>
-      <c r="E18" s="40"/>
+      <c r="E18" s="39"/>
       <c r="F18" s="19"/>
       <c r="H18" s="14"/>
       <c r="I18" s="11"/>
@@ -2190,7 +2278,7 @@
       <c r="L18" s="14"/>
       <c r="M18" s="11"/>
     </row>
-    <row r="19" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D19" s="12"/>
       <c r="E19" s="13"/>
       <c r="H19" s="9"/>
@@ -2200,39 +2288,39 @@
       <c r="L19" s="14"/>
       <c r="M19" s="11"/>
     </row>
-    <row r="20" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C20" s="4"/>
-      <c r="D20" s="46" t="s">
+      <c r="D20" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="E20" s="47"/>
-      <c r="F20" s="41" t="s">
+      <c r="E20" s="41"/>
+      <c r="F20" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="G20" s="43"/>
-      <c r="H20" s="44" t="s">
+      <c r="G20" s="45"/>
+      <c r="H20" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="I20" s="45"/>
+      <c r="I20" s="43"/>
       <c r="J20" s="16"/>
       <c r="K20" s="11"/>
       <c r="L20" s="14"/>
       <c r="M20" s="11"/>
     </row>
-    <row r="21" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C21" s="4"/>
       <c r="D21" s="38"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="41"/>
-      <c r="G21" s="43"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="44"/>
+      <c r="G21" s="45"/>
       <c r="H21" s="38"/>
-      <c r="I21" s="40"/>
+      <c r="I21" s="39"/>
       <c r="J21" s="16"/>
       <c r="K21" s="11"/>
       <c r="L21" s="14"/>
       <c r="M21" s="11"/>
     </row>
-    <row r="22" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D22" s="12"/>
       <c r="E22" s="13"/>
       <c r="H22" s="20"/>
@@ -2242,27 +2330,27 @@
       <c r="L22" s="9"/>
       <c r="M22" s="7"/>
     </row>
-    <row r="23" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C23" s="4"/>
-      <c r="D23" s="46" t="s">
+      <c r="D23" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="E23" s="47"/>
+      <c r="E23" s="41"/>
       <c r="F23" s="8"/>
       <c r="G23" s="21"/>
       <c r="H23" s="21"/>
       <c r="I23" s="21"/>
       <c r="J23" s="9"/>
       <c r="K23" s="17"/>
-      <c r="L23" s="44" t="s">
+      <c r="L23" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="M23" s="45"/>
-    </row>
-    <row r="24" spans="1:13" ht="113.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M23" s="43"/>
+    </row>
+    <row r="24" spans="1:13" ht="113.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C24" s="4"/>
       <c r="D24" s="38"/>
-      <c r="E24" s="40"/>
+      <c r="E24" s="39"/>
       <c r="F24" s="5"/>
       <c r="G24" s="10"/>
       <c r="H24" s="10"/>
@@ -2270,9 +2358,9 @@
       <c r="J24" s="6"/>
       <c r="K24" s="22"/>
       <c r="L24" s="38"/>
-      <c r="M24" s="40"/>
-    </row>
-    <row r="25" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M24" s="39"/>
+    </row>
+    <row r="25" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D25" s="12"/>
       <c r="E25" s="13"/>
       <c r="J25" s="14"/>
@@ -2280,32 +2368,32 @@
       <c r="L25" s="6"/>
       <c r="M25" s="19"/>
     </row>
-    <row r="26" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="3"/>
       <c r="C26" s="23"/>
-      <c r="D26" s="44" t="s">
+      <c r="D26" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="E26" s="45"/>
+      <c r="E26" s="43"/>
       <c r="F26" s="11"/>
       <c r="J26" s="14"/>
       <c r="K26" s="11"/>
       <c r="L26" s="14"/>
       <c r="M26" s="11"/>
     </row>
-    <row r="27" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
       <c r="B27" s="5"/>
       <c r="C27" s="6"/>
       <c r="D27" s="38"/>
-      <c r="E27" s="40"/>
+      <c r="E27" s="39"/>
       <c r="F27" s="11"/>
       <c r="J27" s="14"/>
       <c r="K27" s="11"/>
       <c r="L27" s="14"/>
       <c r="M27" s="11"/>
     </row>
-    <row r="28" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="23"/>
       <c r="B28" s="8"/>
       <c r="D28" s="12"/>
@@ -2315,16 +2403,16 @@
       <c r="L28" s="14"/>
       <c r="M28" s="11"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A29" s="44" t="s">
+    <row r="29" spans="1:13" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A29" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="B29" s="45"/>
+      <c r="B29" s="43"/>
       <c r="C29" s="24"/>
-      <c r="D29" s="46" t="s">
+      <c r="D29" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="47"/>
+      <c r="E29" s="41"/>
       <c r="F29" s="8"/>
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
@@ -2334,12 +2422,12 @@
       <c r="L29" s="14"/>
       <c r="M29" s="11"/>
     </row>
-    <row r="30" spans="1:13" ht="322.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13" ht="322.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="38"/>
-      <c r="B30" s="40"/>
+      <c r="B30" s="39"/>
       <c r="C30" s="24"/>
       <c r="D30" s="38"/>
-      <c r="E30" s="40"/>
+      <c r="E30" s="39"/>
       <c r="F30" s="19"/>
       <c r="G30" s="20"/>
       <c r="H30" s="20"/>
@@ -2348,7 +2436,7 @@
       <c r="L30" s="14"/>
       <c r="M30" s="11"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:13" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A31" s="12"/>
       <c r="B31" s="13"/>
       <c r="D31" s="12"/>
@@ -2356,47 +2444,47 @@
       <c r="L31" s="9"/>
       <c r="M31" s="7"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A32" s="46" t="s">
+    <row r="32" spans="1:13" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A32" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="B32" s="47"/>
+      <c r="B32" s="41"/>
       <c r="C32" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="46" t="s">
+      <c r="D32" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="E32" s="47"/>
-      <c r="F32" s="41" t="s">
+      <c r="E32" s="41"/>
+      <c r="F32" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="G32" s="42"/>
-      <c r="H32" s="42"/>
-      <c r="I32" s="42"/>
-      <c r="J32" s="42"/>
-      <c r="K32" s="43"/>
-      <c r="L32" s="46" t="s">
+      <c r="G32" s="47"/>
+      <c r="H32" s="47"/>
+      <c r="I32" s="47"/>
+      <c r="J32" s="47"/>
+      <c r="K32" s="45"/>
+      <c r="L32" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="M32" s="47"/>
-    </row>
-    <row r="33" spans="1:13" ht="394.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M32" s="41"/>
+    </row>
+    <row r="33" spans="1:13" ht="394.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="48"/>
-      <c r="B33" s="39"/>
+      <c r="B33" s="46"/>
       <c r="C33" s="16"/>
       <c r="D33" s="38"/>
-      <c r="E33" s="40"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="42"/>
-      <c r="H33" s="42"/>
-      <c r="I33" s="42"/>
-      <c r="J33" s="42"/>
-      <c r="K33" s="43"/>
+      <c r="E33" s="39"/>
+      <c r="F33" s="44"/>
+      <c r="G33" s="47"/>
+      <c r="H33" s="47"/>
+      <c r="I33" s="47"/>
+      <c r="J33" s="47"/>
+      <c r="K33" s="45"/>
       <c r="L33" s="38"/>
-      <c r="M33" s="39"/>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M33" s="46"/>
+    </row>
+    <row r="34" spans="1:13" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A34" s="20"/>
       <c r="B34" s="20"/>
       <c r="D34" s="12"/>
@@ -2404,35 +2492,48 @@
       <c r="L34" s="20"/>
       <c r="M34" s="20"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:13" ht="13.2" x14ac:dyDescent="0.25">
       <c r="C35" s="4"/>
-      <c r="D35" s="44" t="s">
+      <c r="D35" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="E35" s="45"/>
+      <c r="E35" s="43"/>
       <c r="F35" s="11"/>
     </row>
-    <row r="36" spans="1:13" ht="213.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:13" ht="213.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C36" s="4"/>
       <c r="D36" s="38"/>
-      <c r="E36" s="40"/>
+      <c r="E36" s="39"/>
       <c r="F36" s="11"/>
     </row>
-    <row r="38" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E38" s="25"/>
       <c r="F38" s="25"/>
       <c r="H38" s="38"/>
-      <c r="I38" s="39"/>
-    </row>
-    <row r="91" ht="0.75" customHeight="1" x14ac:dyDescent="0.2"/>
+      <c r="I38" s="46"/>
+    </row>
+    <row r="91" ht="0.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="F32:K32"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="F33:K33"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="L23:M23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="L32:M32"/>
+    <mergeCell ref="L33:M33"/>
     <mergeCell ref="H20:I20"/>
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="H11:I11"/>
@@ -2449,25 +2550,12 @@
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="D23:E23"/>
-    <mergeCell ref="L23:M23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="L24:M24"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="L32:M32"/>
-    <mergeCell ref="L33:M33"/>
-    <mergeCell ref="H38:I38"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="F32:K32"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="F33:K33"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D8:E8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2479,9 +2567,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43DB12A5-2734-4A80-B355-23ECE7ADE458}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2491,7 +2579,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EA4FA80-9370-4F95-8930-41199F5C753B}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>